<commit_message>
day4: 交易模型拆解 + L1提示词初稿（JSON Schema/evidence）
</commit_message>
<xml_diff>
--- a/plans/AI产品经理学习实践计划表.xlsx
+++ b/plans/AI产品经理学习实践计划表.xlsx
@@ -1645,12 +1645,12 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>★ 集中推进：Figma 装好画 1 页框线；建简历骨架（一页纸）</t>
+          <t>俞军第3部分交易模型 + L1提示词初稿（JSON Schema/evidence）</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>课程 / 开源项目源码阅读</t>
+          <t>L1提示词初稿：3个模板 + 结构化输出 + 证据约束</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>✓</t>
         </is>
       </c>
     </row>

</xml_diff>